<commit_message>
UPDATE: Adds documentation, fixes and test case
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/TEXT/ENCODEURL.xlsx
+++ b/xlsx/tests/calc_tests/TEXT/ENCODEURL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elsam\Downloads\Telegram Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\elsa\IronCalc\xlsx\tests\calc_tests\TEXT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D7F1754-B9E8-491C-9E09-BFBE13629551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9167B78E-42AA-4554-BA78-27D469009D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t>NOTES</t>
   </si>
@@ -100,12 +100,6 @@
   </si>
   <si>
     <t>Uppercase letters and digits (unreserved)</t>
-  </si>
-  <si>
-    <t>-_.~</t>
-  </si>
-  <si>
-    <t>RFC 3986 unreserved punctuation</t>
   </si>
   <si>
     <t>!*'()</t>
@@ -722,7 +716,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B150EF-5E2D-EF45-9F06-93CFDF3000CF}">
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="3" width="43.33203125" customWidth="1"/>
@@ -760,7 +754,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="4" t="str">
-        <f t="shared" ref="B3:B42" si="0">_xlfn.ENCODEURL(A3)</f>
+        <f t="shared" ref="B3:B41" si="0">_xlfn.ENCODEURL(A3)</f>
         <v>hello%20world</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -800,12 +794,14 @@
       </c>
       <c r="B6" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>-_.%7E</v>
+        <v>%21%2A%27%28%29</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="6" t="s">
@@ -813,14 +809,12 @@
       </c>
       <c r="B7" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%21%2A%27%28%29</v>
+        <v>%3B%3A%40%26%3D%2B%24%2C%2F%3F%23%5B%5D</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>73</v>
-      </c>
+      <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" s="6" t="s">
@@ -828,7 +822,7 @@
       </c>
       <c r="B8" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%3B%3A%40%26%3D%2B%24%2C%2F%3F%23%5B%5D</v>
+        <v>%25</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>20</v>
@@ -841,7 +835,7 @@
       </c>
       <c r="B9" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%25</v>
+        <v>a%2520b</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>22</v>
@@ -854,7 +848,7 @@
       </c>
       <c r="B10" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>a%2520b</v>
+        <v>a%2Bb</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>24</v>
@@ -867,7 +861,7 @@
       </c>
       <c r="B11" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>a%2Bb</v>
+        <v>a%20%20b</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>26</v>
@@ -880,7 +874,7 @@
       </c>
       <c r="B12" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>a%20%20b</v>
+        <v>%20x%20</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>28</v>
@@ -888,84 +882,84 @@
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="6" t="str">
+        <f>"a"&amp;CHAR(9)&amp;"b"</f>
+        <v>a	b</v>
+      </c>
+      <c r="B13" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>a%09b</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B13" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>%20x%20</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="6" t="str">
-        <f>"a"&amp;CHAR(9)&amp;"b"</f>
-        <v>a	b</v>
-      </c>
-      <c r="B14" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>a%09b</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A15" s="6" t="str">
         <f>"a"&amp;CHAR(10)&amp;"b"</f>
         <v>a
 b</v>
       </c>
-      <c r="B15" s="4" t="str">
+      <c r="B14" s="4" t="str">
         <f t="shared" si="0"/>
         <v>a%0Ab</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A16" s="6" t="str">
+      <c r="C14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A15" s="6" t="str">
         <f>"a"&amp;CHAR(13)&amp;CHAR(10)&amp;"b"</f>
         <v>a_x000D_
 b</v>
       </c>
+      <c r="B15" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>a%0D%0Ab</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A16" s="6" t="str">
+        <f>CHAR(1)</f>
+        <v>_x0001_</v>
+      </c>
       <c r="B16" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>a%0D%0Ab</v>
+        <v>%01</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="str">
-        <f>CHAR(1)</f>
-        <v>_x0001_</v>
-      </c>
-      <c r="B17" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>%01</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A18" s="6" t="str">
         <f>CHAR(34)</f>
         <v>"</v>
       </c>
+      <c r="B17" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>%22</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A18" s="6" t="s">
+        <v>34</v>
+      </c>
       <c r="B18" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%22</v>
+        <v>%3C%3E</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>35</v>
@@ -978,7 +972,7 @@
       </c>
       <c r="B19" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%3C%3E</v>
+        <v>%5C%7C%5E%60%7B%7D</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>37</v>
@@ -986,82 +980,82 @@
       <c r="D19" s="1"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="6" t="str">
+        <f>_xlfn.UNICHAR(233)</f>
+        <v>é</v>
+      </c>
+      <c r="B20" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>%C3%A9</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B20" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>%5C%7C%5E%60%7B%7D</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D20" s="1"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="6" t="str">
-        <f>_xlfn.UNICHAR(233)</f>
-        <v>é</v>
+        <f>_xlfn.UNICHAR(252)&amp;"ber"</f>
+        <v>über</v>
       </c>
       <c r="B21" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%C3%A9</v>
+        <v>%C3%BCber</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D21" s="1"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" s="6" t="str">
-        <f>_xlfn.UNICHAR(252)&amp;"ber"</f>
-        <v>über</v>
+        <f>_xlfn.UNICHAR(8364)</f>
+        <v>€</v>
       </c>
       <c r="B22" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%C3%BCber</v>
+        <v>%E2%82%AC</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D22" s="1"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="6" t="str">
-        <f>_xlfn.UNICHAR(8364)</f>
-        <v>€</v>
+        <f>_xlfn.UNICHAR(26085)&amp;_xlfn.UNICHAR(26412)</f>
+        <v>日本</v>
       </c>
       <c r="B23" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%E2%82%AC</v>
+        <v>%E6%97%A5%E6%9C%AC</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D23" s="1"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="6" t="str">
-        <f>_xlfn.UNICHAR(26085)&amp;_xlfn.UNICHAR(26412)</f>
-        <v>日本</v>
-      </c>
-      <c r="B24" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>%E6%97%A5%E6%9C%AC</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A25" s="6" t="str">
         <f>_xlfn.UNICHAR(128512)</f>
         <v>😀</v>
       </c>
+      <c r="B24" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>%F0%9F%98%80</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="1"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A25" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="B25" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>%F0%9F%98%80</v>
+        <v>https%3A%2F%2Fexample.com%2Fsearch%3Fq%3Da%20b%26lang%3Den</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>44</v>
@@ -1069,349 +1063,336 @@
       <c r="D25" s="1"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A26" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B26" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>https%3A%2F%2Fexample.com%2Fsearch%3Fq%3Da%20b%26lang%3Den</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D26" s="1"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A27" s="6" t="str">
+      <c r="A26" s="6" t="str">
         <f>""</f>
         <v/>
       </c>
+      <c r="B26" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D26" s="1"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A27" s="6"/>
       <c r="B27" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C27" s="1" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="D27" s="1"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A28" s="6"/>
+      <c r="A28" s="6">
+        <v>123</v>
+      </c>
       <c r="B28" s="4" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>123</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D28" s="1"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="6">
-        <v>123</v>
+        <v>3.14</v>
       </c>
       <c r="B29" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>123</v>
+        <v>3.14</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D29" s="1"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" s="6">
-        <v>3.14</v>
+        <v>-5</v>
       </c>
       <c r="B30" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>3.14</v>
+        <v>-5</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D30" s="1"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="6">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="B31" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31" s="1"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A32" s="7">
+        <v>1E+20</v>
+      </c>
+      <c r="B32" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>1E%2B20</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="D31" s="1"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A32" s="6">
-        <v>0</v>
-      </c>
-      <c r="B32" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="D32" s="1"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="7">
-        <v>1E+20</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="B33" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>1E%2B20</v>
+        <v>0.0000001</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D33" s="1"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A34" s="7">
-        <v>9.9999999999999995E-8</v>
-      </c>
-      <c r="B34" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>0.0000001</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D34" s="1"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A35" s="6">
+      <c r="A34" s="6">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
+      <c r="B34" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>0.333333333333333</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" s="1"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A35" s="6" t="b">
+        <v>1</v>
+      </c>
       <c r="B35" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>0.333333333333333</v>
+        <v>TRUE</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D35" s="1"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="B36" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>FALSE</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D36" s="1"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A37" s="8">
+        <v>46040</v>
+      </c>
+      <c r="B37" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>46040</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D37" s="1"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A38" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="B38" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" s="1"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A39" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B36" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>TRUE</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D36" s="1"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A37" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="B37" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>FALSE</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D37" s="1"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A38" s="8">
-        <v>46040</v>
-      </c>
-      <c r="B38" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>46040</v>
-      </c>
-      <c r="C38" s="1" t="s">
+      <c r="B39" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D38" s="1"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A39" s="9">
-        <v>0.5</v>
-      </c>
-      <c r="B39" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="D39" s="1"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A40" s="6" t="e">
+        <f>1/0</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="B40" s="4" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="D39" s="1"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A40" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="B40" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>100</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="D40" s="1"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="6" t="e">
-        <f>1/0</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="B41" s="4" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D41" s="1"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A42" s="6" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="B42" s="4" t="e">
+      <c r="B41" s="4" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
+      <c r="C41" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D41" s="1"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A42" s="6"/>
+      <c r="B42" s="5" t="str">
+        <f>_xlfn.ENCODEURL("a b")</f>
+        <v>a%20b</v>
+      </c>
       <c r="C42" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D42" s="1"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A43" s="6"/>
       <c r="B43" s="5" t="str">
-        <f>_xlfn.ENCODEURL("a b")</f>
-        <v>a%20b</v>
+        <f>_xlfn.ENCODEURL(1.5)</f>
+        <v>1.5</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D43" s="1"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" s="6"/>
       <c r="B44" s="5" t="str">
-        <f>_xlfn.ENCODEURL(1.5)</f>
-        <v>1.5</v>
+        <f>_xlfn.ENCODEURL(TRUE)</f>
+        <v>TRUE</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D44" s="1"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A45" s="6"/>
       <c r="B45" s="5" t="str">
-        <f>_xlfn.ENCODEURL(TRUE)</f>
-        <v>TRUE</v>
+        <f>_xlfn.ENCODEURL("")</f>
+        <v/>
       </c>
       <c r="C45" s="1" t="s">
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="D45" s="1"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A46" s="6"/>
       <c r="B46" s="5" t="str">
-        <f>_xlfn.ENCODEURL("")</f>
-        <v/>
+        <f>_xlfn.ENCODEURL("x"&amp;"y z")</f>
+        <v>xy%20z</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="D46" s="1"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A47" s="6"/>
       <c r="B47" s="5" t="str">
-        <f>_xlfn.ENCODEURL("x"&amp;"y z")</f>
-        <v>xy%20z</v>
+        <f>_xlfn.ENCODEURL(_xlfn.ENCODEURL("a b"))</f>
+        <v>a%2520b</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D47" s="1"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A48" s="6"/>
-      <c r="B48" s="5" t="str">
-        <f>_xlfn.ENCODEURL(_xlfn.ENCODEURL("a b"))</f>
-        <v>a%2520b</v>
+      <c r="B48" s="5" t="e">
+        <f>LEN(_xlfn.ENCODEURL(REPT("a",32767)))</f>
+        <v>#VALUE!</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D48" s="1"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A49" s="6"/>
-      <c r="B49" s="5" t="e">
-        <f>LEN(_xlfn.ENCODEURL(REPT("a",32767)))</f>
-        <v>#VALUE!</v>
+      <c r="B49" s="5">
+        <f>LEN(_xlfn.ENCODEURL(REPT(" ",10922)))</f>
+        <v>32766</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D49" s="1"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A50" s="6"/>
-      <c r="B50" s="5">
-        <f>LEN(_xlfn.ENCODEURL(REPT(" ",10922)))</f>
-        <v>32766</v>
+      <c r="B50" s="5" t="e">
+        <f>_xlfn.ENCODEURL(REPT(" ",10923))</f>
+        <v>#VALUE!</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D50" s="1"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A51" s="6"/>
-      <c r="B51" s="5" t="e">
-        <f>_xlfn.ENCODEURL(REPT(" ",10923))</f>
-        <v>#VALUE!</v>
+      <c r="B51" s="5" t="str" cm="1">
+        <f t="array" ref="B51">INDEX(_xlfn.ENCODEURL(A2:A4),2)</f>
+        <v>hello%20world</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D51" s="1"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A52" s="6"/>
-      <c r="B52" s="5" t="str" cm="1">
-        <f t="array" ref="B52">INDEX(_xlfn.ENCODEURL(A2:A4),2)</f>
-        <v>hello%20world</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D52" s="1"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A53" s="6"/>
-      <c r="B53" s="5" t="str">
+      <c r="B52" s="5" t="str">
         <f>_xlfn.ENCODEURL(D:D)</f>
         <v>a%20b%2Fc</v>
       </c>
-      <c r="C53" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>72</v>
+      <c r="C52" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>